<commit_message>
Update latency measurement spreadsheet and README for version 2.1.0
</commit_message>
<xml_diff>
--- a/docs/Latency per message v 2.1.0.xlsx
+++ b/docs/Latency per message v 2.1.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\whghk\Desktop\Coding\Intellij\embellish_chat\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F41866FA-BD44-4D73-B0BC-DAFE4595A952}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0976AB2C-8268-4807-A85E-A71036C16B24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{30AE5353-CC8E-4A31-864B-BE4B1A53EFC5}"/>
   </bookViews>
@@ -42,15 +42,15 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>v2.1.0/min</t>
+    <t>min</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>v2.1.0/avg</t>
+    <t>avg</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>v2.1.0/max</t>
+    <t>max</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>

</xml_diff>